<commit_message>
#112 safety_specs.xslx replace ITTFL by SAFFL in ADVS dataset. ITTFL is not available anymore in pharmaverseadam::adsl.
</commit_message>
<xml_diff>
--- a/metadata/safety_specs.xlsx
+++ b/metadata/safety_specs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Fanny.Gautier\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A063C20B-47FA-426E-A1CB-54C3717EE6BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44FF1EC9-6EB9-4428-B2F7-0ABEE050E695}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28800" windowHeight="14535" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38400" windowHeight="19815" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Study" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2082" uniqueCount="694">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2082" uniqueCount="693">
   <si>
     <t>Attribute</t>
   </si>
@@ -1219,9 +1219,6 @@
   </si>
   <si>
     <t>ADSL.RACE</t>
-  </si>
-  <si>
-    <t>ADSL.ITTFL</t>
   </si>
   <si>
     <t>VS.DOMAIN</t>
@@ -2702,7 +2699,7 @@
         <v>41</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="30" x14ac:dyDescent="0.25">
@@ -2710,7 +2707,7 @@
         <v>42</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -2898,20 +2895,20 @@
     </row>
     <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B4" s="17" t="s">
+        <v>632</v>
+      </c>
+      <c r="C4" s="17" t="s">
         <v>633</v>
-      </c>
-      <c r="C4" s="17" t="s">
-        <v>634</v>
       </c>
       <c r="D4" s="8"/>
       <c r="E4" s="13" t="s">
         <v>48</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="G4" s="17" t="s">
         <v>200</v>
@@ -3327,7 +3324,7 @@
         <v>50</v>
       </c>
       <c r="J11" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="K11" t="s">
         <v>85</v>
@@ -3388,7 +3385,7 @@
         <v>49</v>
       </c>
       <c r="J13" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="K13" t="s">
         <v>23</v>
@@ -3423,7 +3420,7 @@
         <v>49</v>
       </c>
       <c r="J14" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="K14" t="s">
         <v>23</v>
@@ -3458,7 +3455,7 @@
         <v>50</v>
       </c>
       <c r="J15" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="K15" t="s">
         <v>268</v>
@@ -3487,7 +3484,7 @@
         <v>50</v>
       </c>
       <c r="J16" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="K16" t="s">
         <v>85</v>
@@ -3519,7 +3516,7 @@
         <v>50</v>
       </c>
       <c r="J17" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="K17" t="s">
         <v>268</v>
@@ -3586,7 +3583,7 @@
         <v>23</v>
       </c>
       <c r="N19" s="12" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="O19" t="s">
         <v>283</v>
@@ -3621,7 +3618,7 @@
         <v>23</v>
       </c>
       <c r="M20" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="N20" s="12"/>
     </row>
@@ -3997,7 +3994,7 @@
         <v>245</v>
       </c>
       <c r="E32" s="22" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="F32">
         <v>8</v>
@@ -4206,10 +4203,10 @@
         <v>215</v>
       </c>
       <c r="C39" t="s">
+        <v>591</v>
+      </c>
+      <c r="D39" t="s">
         <v>592</v>
-      </c>
-      <c r="D39" t="s">
-        <v>593</v>
       </c>
       <c r="E39" t="s">
         <v>84</v>
@@ -4224,7 +4221,7 @@
         <v>23</v>
       </c>
       <c r="N39" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
     </row>
     <row r="40" spans="1:14" customFormat="1" x14ac:dyDescent="0.25">
@@ -4267,10 +4264,10 @@
         <v>215</v>
       </c>
       <c r="C41" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="D41" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="E41" t="s">
         <v>84</v>
@@ -4285,7 +4282,7 @@
         <v>85</v>
       </c>
       <c r="M41" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
     </row>
     <row r="42" spans="1:14" customFormat="1" x14ac:dyDescent="0.25">
@@ -4473,10 +4470,10 @@
         <v>215</v>
       </c>
       <c r="C48" t="s">
+        <v>599</v>
+      </c>
+      <c r="D48" t="s">
         <v>600</v>
-      </c>
-      <c r="D48" t="s">
-        <v>601</v>
       </c>
       <c r="E48" t="s">
         <v>226</v>
@@ -4491,7 +4488,7 @@
         <v>85</v>
       </c>
       <c r="M48" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="49" spans="1:14" customFormat="1" x14ac:dyDescent="0.25">
@@ -4932,7 +4929,7 @@
         <v>49</v>
       </c>
       <c r="J63" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="K63" t="s">
         <v>23</v>
@@ -4964,7 +4961,7 @@
         <v>49</v>
       </c>
       <c r="J64" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="K64" t="s">
         <v>23</v>
@@ -4981,10 +4978,10 @@
         <v>216</v>
       </c>
       <c r="C65" t="s">
-        <v>235</v>
+        <v>124</v>
       </c>
       <c r="D65" t="s">
-        <v>236</v>
+        <v>118</v>
       </c>
       <c r="E65" t="s">
         <v>84</v>
@@ -5002,7 +4999,7 @@
         <v>23</v>
       </c>
       <c r="N65" t="s">
-        <v>386</v>
+        <v>588</v>
       </c>
     </row>
     <row r="66" spans="1:14" customFormat="1" x14ac:dyDescent="0.25">
@@ -5191,7 +5188,7 @@
         <v>23</v>
       </c>
       <c r="N71" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="72" spans="1:14" customFormat="1" x14ac:dyDescent="0.25">
@@ -5220,7 +5217,7 @@
         <v>23</v>
       </c>
       <c r="N72" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="73" spans="1:14" customFormat="1" x14ac:dyDescent="0.25">
@@ -5249,7 +5246,7 @@
         <v>23</v>
       </c>
       <c r="N73" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="74" spans="1:14" customFormat="1" x14ac:dyDescent="0.25">
@@ -5278,7 +5275,7 @@
         <v>23</v>
       </c>
       <c r="N74" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="75" spans="1:14" customFormat="1" x14ac:dyDescent="0.25">
@@ -5307,7 +5304,7 @@
         <v>23</v>
       </c>
       <c r="N75" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="76" spans="1:14" customFormat="1" x14ac:dyDescent="0.25">
@@ -5336,7 +5333,7 @@
         <v>23</v>
       </c>
       <c r="N76" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="77" spans="1:14" customFormat="1" x14ac:dyDescent="0.25">
@@ -5365,7 +5362,7 @@
         <v>23</v>
       </c>
       <c r="N77" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="78" spans="1:14" customFormat="1" x14ac:dyDescent="0.25">
@@ -5394,7 +5391,7 @@
         <v>23</v>
       </c>
       <c r="N78" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="79" spans="1:14" customFormat="1" x14ac:dyDescent="0.25">
@@ -5423,7 +5420,7 @@
         <v>23</v>
       </c>
       <c r="N79" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="80" spans="1:14" customFormat="1" x14ac:dyDescent="0.25">
@@ -5452,7 +5449,7 @@
         <v>23</v>
       </c>
       <c r="N80" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="81" spans="1:14" customFormat="1" x14ac:dyDescent="0.25">
@@ -5481,7 +5478,7 @@
         <v>23</v>
       </c>
       <c r="N81" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="82" spans="1:14" customFormat="1" x14ac:dyDescent="0.25">
@@ -5510,7 +5507,7 @@
         <v>23</v>
       </c>
       <c r="N82" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="83" spans="1:14" customFormat="1" x14ac:dyDescent="0.25">
@@ -5539,7 +5536,7 @@
         <v>23</v>
       </c>
       <c r="N83" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="84" spans="1:14" customFormat="1" x14ac:dyDescent="0.25">
@@ -5568,7 +5565,7 @@
         <v>23</v>
       </c>
       <c r="N84" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="85" spans="1:14" customFormat="1" x14ac:dyDescent="0.25">
@@ -5597,7 +5594,7 @@
         <v>23</v>
       </c>
       <c r="N85" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="86" spans="1:14" customFormat="1" x14ac:dyDescent="0.25">
@@ -5626,7 +5623,7 @@
         <v>23</v>
       </c>
       <c r="N86" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="87" spans="1:14" customFormat="1" x14ac:dyDescent="0.25">
@@ -5655,7 +5652,7 @@
         <v>23</v>
       </c>
       <c r="N87" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="88" spans="1:14" customFormat="1" x14ac:dyDescent="0.25">
@@ -5684,7 +5681,7 @@
         <v>23</v>
       </c>
       <c r="N88" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="89" spans="1:14" customFormat="1" x14ac:dyDescent="0.25">
@@ -5713,7 +5710,7 @@
         <v>23</v>
       </c>
       <c r="N89" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="90" spans="1:14" customFormat="1" x14ac:dyDescent="0.25">
@@ -5742,7 +5739,7 @@
         <v>23</v>
       </c>
       <c r="N90" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="91" spans="1:14" customFormat="1" x14ac:dyDescent="0.25">
@@ -5771,7 +5768,7 @@
         <v>23</v>
       </c>
       <c r="N91" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="92" spans="1:14" customFormat="1" x14ac:dyDescent="0.25">
@@ -5800,7 +5797,7 @@
         <v>23</v>
       </c>
       <c r="N92" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="93" spans="1:14" customFormat="1" x14ac:dyDescent="0.25">
@@ -5913,7 +5910,7 @@
         <v>85</v>
       </c>
       <c r="M96" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="97" spans="1:13" customFormat="1" x14ac:dyDescent="0.25">
@@ -5939,7 +5936,7 @@
         <v>268</v>
       </c>
       <c r="M97" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="98" spans="1:13" customFormat="1" x14ac:dyDescent="0.25">
@@ -5965,7 +5962,7 @@
         <v>85</v>
       </c>
       <c r="M98" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="99" spans="1:13" customFormat="1" x14ac:dyDescent="0.25">
@@ -6014,7 +6011,7 @@
         <v>85</v>
       </c>
       <c r="M100" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="101" spans="1:13" customFormat="1" x14ac:dyDescent="0.25">
@@ -6040,7 +6037,7 @@
         <v>268</v>
       </c>
       <c r="M101" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="102" spans="1:13" customFormat="1" x14ac:dyDescent="0.25">
@@ -6069,7 +6066,7 @@
         <v>85</v>
       </c>
       <c r="M102" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="103" spans="1:13" customFormat="1" x14ac:dyDescent="0.25">
@@ -6095,7 +6092,7 @@
         <v>85</v>
       </c>
       <c r="M103" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="104" spans="1:13" customFormat="1" x14ac:dyDescent="0.25">
@@ -6121,7 +6118,7 @@
         <v>85</v>
       </c>
       <c r="M104" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="105" spans="1:13" customFormat="1" x14ac:dyDescent="0.25">
@@ -6147,7 +6144,7 @@
         <v>85</v>
       </c>
       <c r="M105" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="106" spans="1:13" customFormat="1" x14ac:dyDescent="0.25">
@@ -6173,7 +6170,7 @@
         <v>268</v>
       </c>
       <c r="M106" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="107" spans="1:13" customFormat="1" x14ac:dyDescent="0.25">
@@ -6199,7 +6196,7 @@
         <v>268</v>
       </c>
       <c r="M107" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="108" spans="1:13" customFormat="1" x14ac:dyDescent="0.25">
@@ -6225,7 +6222,7 @@
         <v>85</v>
       </c>
       <c r="M108" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="109" spans="1:13" customFormat="1" x14ac:dyDescent="0.25">
@@ -6251,7 +6248,7 @@
         <v>85</v>
       </c>
       <c r="M109" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="110" spans="1:13" customFormat="1" x14ac:dyDescent="0.25">
@@ -6277,7 +6274,7 @@
         <v>268</v>
       </c>
       <c r="M110" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="111" spans="1:13" customFormat="1" x14ac:dyDescent="0.25">
@@ -6303,7 +6300,7 @@
         <v>268</v>
       </c>
       <c r="M111" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="112" spans="1:13" customFormat="1" x14ac:dyDescent="0.25">
@@ -6329,7 +6326,7 @@
         <v>85</v>
       </c>
       <c r="M112" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="113" spans="1:16" customFormat="1" x14ac:dyDescent="0.25">
@@ -6355,7 +6352,7 @@
         <v>85</v>
       </c>
       <c r="M113" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="114" spans="1:16" customFormat="1" x14ac:dyDescent="0.25">
@@ -6381,7 +6378,7 @@
         <v>85</v>
       </c>
       <c r="M114" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="115" spans="1:16" customFormat="1" x14ac:dyDescent="0.25">
@@ -6407,7 +6404,7 @@
         <v>268</v>
       </c>
       <c r="M115" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="116" spans="1:16" customFormat="1" x14ac:dyDescent="0.25">
@@ -6433,7 +6430,7 @@
         <v>85</v>
       </c>
       <c r="M116" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="117" spans="1:16" customFormat="1" x14ac:dyDescent="0.25">
@@ -6459,7 +6456,7 @@
         <v>268</v>
       </c>
       <c r="M117" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="118" spans="1:16" customFormat="1" x14ac:dyDescent="0.25">
@@ -6485,7 +6482,7 @@
         <v>85</v>
       </c>
       <c r="M118" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="119" spans="1:16" customFormat="1" x14ac:dyDescent="0.25">
@@ -6511,7 +6508,7 @@
         <v>85</v>
       </c>
       <c r="M119" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="120" spans="1:16" customFormat="1" x14ac:dyDescent="0.25">
@@ -6540,7 +6537,7 @@
         <v>85</v>
       </c>
       <c r="M120" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="121" spans="1:16" customFormat="1" x14ac:dyDescent="0.25">
@@ -6569,7 +6566,7 @@
         <v>85</v>
       </c>
       <c r="M121" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="122" spans="1:16" x14ac:dyDescent="0.25">
@@ -6577,7 +6574,7 @@
         <v>1</v>
       </c>
       <c r="B122" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C122" t="s">
         <v>51</v>
@@ -6613,7 +6610,7 @@
         <v>2</v>
       </c>
       <c r="B123" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C123" t="s">
         <v>52</v>
@@ -6649,7 +6646,7 @@
         <v>3</v>
       </c>
       <c r="B124" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C124" t="s">
         <v>55</v>
@@ -6685,7 +6682,7 @@
         <v>4</v>
       </c>
       <c r="B125" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C125" t="s">
         <v>57</v>
@@ -6721,7 +6718,7 @@
         <v>5</v>
       </c>
       <c r="B126" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C126" t="s">
         <v>144</v>
@@ -6757,7 +6754,7 @@
         <v>6</v>
       </c>
       <c r="B127" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C127" t="s">
         <v>67</v>
@@ -6793,7 +6790,7 @@
         <v>7</v>
       </c>
       <c r="B128" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C128" t="s">
         <v>62</v>
@@ -6829,7 +6826,7 @@
         <v>8</v>
       </c>
       <c r="B129" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C129" t="s">
         <v>58</v>
@@ -6865,7 +6862,7 @@
         <v>9</v>
       </c>
       <c r="B130" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C130" t="s">
         <v>59</v>
@@ -6901,7 +6898,7 @@
         <v>10</v>
       </c>
       <c r="B131" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C131" t="s">
         <v>60</v>
@@ -6921,7 +6918,7 @@
         <v>49</v>
       </c>
       <c r="J131" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="K131" t="s">
         <v>23</v>
@@ -6939,7 +6936,7 @@
         <v>11</v>
       </c>
       <c r="B132" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C132" t="s">
         <v>61</v>
@@ -6959,7 +6956,7 @@
         <v>49</v>
       </c>
       <c r="J132" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="K132" t="s">
         <v>23</v>
@@ -6977,7 +6974,7 @@
         <v>12</v>
       </c>
       <c r="B133" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C133" t="s">
         <v>127</v>
@@ -7015,7 +7012,7 @@
         <v>13</v>
       </c>
       <c r="B134" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C134" t="s">
         <v>129</v>
@@ -7053,7 +7050,7 @@
         <v>14</v>
       </c>
       <c r="B135" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C135" t="s">
         <v>138</v>
@@ -7091,7 +7088,7 @@
         <v>15</v>
       </c>
       <c r="B136" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C136" t="s">
         <v>131</v>
@@ -7129,7 +7126,7 @@
         <v>16</v>
       </c>
       <c r="B137" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C137" t="s">
         <v>140</v>
@@ -7167,7 +7164,7 @@
         <v>17</v>
       </c>
       <c r="B138" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C138" t="s">
         <v>124</v>
@@ -7193,7 +7190,7 @@
       <c r="L138"/>
       <c r="M138"/>
       <c r="N138" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="O138"/>
       <c r="P138"/>
@@ -7203,7 +7200,7 @@
         <v>18</v>
       </c>
       <c r="B139" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C139" t="s">
         <v>250</v>
@@ -7241,7 +7238,7 @@
         <v>19</v>
       </c>
       <c r="B140" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C140" t="s">
         <v>66</v>
@@ -7262,7 +7259,7 @@
         <v>23</v>
       </c>
       <c r="N140" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
     <row r="141" spans="1:16" x14ac:dyDescent="0.25">
@@ -7270,10 +7267,10 @@
         <v>20</v>
       </c>
       <c r="B141" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C141" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="D141" t="s">
         <v>342</v>
@@ -7296,7 +7293,7 @@
       <c r="L141"/>
       <c r="M141" s="11"/>
       <c r="N141" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="O141"/>
       <c r="P141"/>
@@ -7306,13 +7303,13 @@
         <v>21</v>
       </c>
       <c r="B142" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C142" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="D142" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="E142" t="s">
         <v>84</v>
@@ -7332,7 +7329,7 @@
       <c r="L142"/>
       <c r="M142" s="11"/>
       <c r="N142" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="O142"/>
       <c r="P142"/>
@@ -7342,13 +7339,13 @@
         <v>22</v>
       </c>
       <c r="B143" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C143" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="D143" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="E143" t="s">
         <v>84</v>
@@ -7368,7 +7365,7 @@
       <c r="L143"/>
       <c r="M143" s="11"/>
       <c r="N143" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="O143"/>
       <c r="P143"/>
@@ -7378,13 +7375,13 @@
         <v>23</v>
       </c>
       <c r="B144" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C144" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="D144" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="E144" t="s">
         <v>84</v>
@@ -7404,7 +7401,7 @@
       <c r="L144"/>
       <c r="M144" s="11"/>
       <c r="N144" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="O144"/>
       <c r="P144"/>
@@ -7414,13 +7411,13 @@
         <v>24</v>
       </c>
       <c r="B145" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C145" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="D145" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="E145" t="s">
         <v>84</v>
@@ -7440,7 +7437,7 @@
       <c r="L145"/>
       <c r="M145" s="11"/>
       <c r="N145" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="O145"/>
       <c r="P145"/>
@@ -7450,13 +7447,13 @@
         <v>25</v>
       </c>
       <c r="B146" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C146" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="D146" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="E146" t="s">
         <v>84</v>
@@ -7476,7 +7473,7 @@
       <c r="L146"/>
       <c r="M146" s="11"/>
       <c r="N146" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="O146"/>
       <c r="P146"/>
@@ -7486,13 +7483,13 @@
         <v>26</v>
       </c>
       <c r="B147" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C147" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="D147" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="E147" t="s">
         <v>84</v>
@@ -7512,7 +7509,7 @@
       <c r="L147"/>
       <c r="M147" s="11"/>
       <c r="N147" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="O147"/>
       <c r="P147"/>
@@ -7522,13 +7519,13 @@
         <v>27</v>
       </c>
       <c r="B148" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C148" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="D148" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="E148" t="s">
         <v>84</v>
@@ -7548,7 +7545,7 @@
       <c r="L148"/>
       <c r="M148" s="11"/>
       <c r="N148" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="O148"/>
       <c r="P148"/>
@@ -7558,13 +7555,13 @@
         <v>28</v>
       </c>
       <c r="B149" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C149" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="D149" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="E149" t="s">
         <v>84</v>
@@ -7584,7 +7581,7 @@
       <c r="L149"/>
       <c r="M149" s="11"/>
       <c r="N149" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="O149"/>
       <c r="P149"/>
@@ -7594,13 +7591,13 @@
         <v>29</v>
       </c>
       <c r="B150" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C150" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="D150" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="E150" t="s">
         <v>84</v>
@@ -7620,7 +7617,7 @@
       <c r="L150"/>
       <c r="M150" s="11"/>
       <c r="N150" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="O150"/>
       <c r="P150"/>
@@ -7630,13 +7627,13 @@
         <v>30</v>
       </c>
       <c r="B151" t="s">
+        <v>605</v>
+      </c>
+      <c r="C151" s="12" t="s">
         <v>606</v>
       </c>
-      <c r="C151" s="12" t="s">
-        <v>607</v>
-      </c>
       <c r="D151" s="12" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="E151" t="s">
         <v>226</v>
@@ -7655,7 +7652,7 @@
         <v>85</v>
       </c>
       <c r="M151" s="12" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
     </row>
     <row r="152" spans="1:16" x14ac:dyDescent="0.25">
@@ -7663,13 +7660,13 @@
         <v>31</v>
       </c>
       <c r="B152" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C152" s="12" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="D152" s="12" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="E152" s="12" t="s">
         <v>84</v>
@@ -7684,7 +7681,7 @@
         <v>85</v>
       </c>
       <c r="M152" s="12" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
     </row>
     <row r="153" spans="1:16" x14ac:dyDescent="0.25">
@@ -7692,13 +7689,13 @@
         <v>32</v>
       </c>
       <c r="B153" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C153" s="12" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="D153" s="12" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="E153" t="s">
         <v>226</v>
@@ -7713,7 +7710,7 @@
         <v>85</v>
       </c>
       <c r="M153" s="12" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
     </row>
     <row r="154" spans="1:16" x14ac:dyDescent="0.25">
@@ -7721,13 +7718,13 @@
         <v>33</v>
       </c>
       <c r="B154" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C154" s="12" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="D154" s="12" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="E154" t="s">
         <v>226</v>
@@ -7746,7 +7743,7 @@
         <v>85</v>
       </c>
       <c r="M154" s="12" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
     </row>
     <row r="155" spans="1:16" x14ac:dyDescent="0.25">
@@ -7754,13 +7751,13 @@
         <v>34</v>
       </c>
       <c r="B155" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C155" s="12" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="D155" s="12" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="E155" s="12" t="s">
         <v>84</v>
@@ -7775,7 +7772,7 @@
         <v>85</v>
       </c>
       <c r="M155" s="12" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
     </row>
     <row r="156" spans="1:16" x14ac:dyDescent="0.25">
@@ -7783,13 +7780,13 @@
         <v>35</v>
       </c>
       <c r="B156" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C156" s="12" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="D156" s="12" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="E156" t="s">
         <v>226</v>
@@ -7804,7 +7801,7 @@
         <v>85</v>
       </c>
       <c r="M156" s="12" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
     </row>
     <row r="157" spans="1:16" x14ac:dyDescent="0.25">
@@ -7812,13 +7809,13 @@
         <v>36</v>
       </c>
       <c r="B157" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C157" s="12" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="D157" s="12" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="E157" t="s">
         <v>226</v>
@@ -7833,7 +7830,7 @@
         <v>85</v>
       </c>
       <c r="M157" s="12" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
     </row>
     <row r="158" spans="1:16" x14ac:dyDescent="0.25">
@@ -7841,13 +7838,13 @@
         <v>37</v>
       </c>
       <c r="B158" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C158" s="12" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="D158" s="12" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="E158" t="s">
         <v>84</v>
@@ -7862,7 +7859,7 @@
         <v>85</v>
       </c>
       <c r="M158" s="12" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
     </row>
     <row r="159" spans="1:16" x14ac:dyDescent="0.25">
@@ -7870,13 +7867,13 @@
         <v>38</v>
       </c>
       <c r="B159" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C159" s="12" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="D159" s="12" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="E159" t="s">
         <v>226</v>
@@ -7895,21 +7892,21 @@
         <v>85</v>
       </c>
       <c r="M159" s="12" t="s">
-        <v>627</v>
-      </c>
-    </row>
-    <row r="160" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="160" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A160">
         <v>39</v>
       </c>
       <c r="B160" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C160" s="12" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="D160" s="12" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="E160" s="12" t="s">
         <v>84</v>
@@ -7924,7 +7921,7 @@
         <v>85</v>
       </c>
       <c r="M160" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="161" spans="1:13" x14ac:dyDescent="0.25">
@@ -7932,13 +7929,13 @@
         <v>40</v>
       </c>
       <c r="B161" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C161" s="12" t="s">
         <v>368</v>
       </c>
       <c r="D161" s="12" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="E161" s="12" t="s">
         <v>84</v>
@@ -7953,7 +7950,7 @@
         <v>85</v>
       </c>
       <c r="M161" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
     </row>
     <row r="162" spans="1:13" x14ac:dyDescent="0.25">
@@ -7961,13 +7958,13 @@
         <v>41</v>
       </c>
       <c r="B162" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C162" s="12" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="D162" s="12" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="E162" s="12" t="s">
         <v>84</v>
@@ -7982,7 +7979,7 @@
         <v>85</v>
       </c>
       <c r="M162" s="12" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
     </row>
     <row r="163" spans="1:13" x14ac:dyDescent="0.25">
@@ -7990,19 +7987,19 @@
         <v>42</v>
       </c>
       <c r="B163" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C163" s="12" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="D163" s="12" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="E163" s="12" t="s">
         <v>84</v>
       </c>
       <c r="F163" s="12" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="I163" t="s">
         <v>49</v>
@@ -8011,7 +8008,7 @@
         <v>85</v>
       </c>
       <c r="M163" s="12" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
     </row>
     <row r="164" spans="1:13" x14ac:dyDescent="0.25">
@@ -8019,19 +8016,19 @@
         <v>43</v>
       </c>
       <c r="B164" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C164" s="12" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="D164" s="12" t="s">
+        <v>670</v>
+      </c>
+      <c r="E164" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="F164" s="12" t="s">
         <v>671</v>
-      </c>
-      <c r="E164" s="12" t="s">
-        <v>84</v>
-      </c>
-      <c r="F164" s="12" t="s">
-        <v>672</v>
       </c>
       <c r="I164" t="s">
         <v>49</v>
@@ -8040,7 +8037,7 @@
         <v>85</v>
       </c>
       <c r="M164" s="12" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
     </row>
   </sheetData>
@@ -8209,7 +8206,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="B2" s="18" t="s">
         <v>228</v>
@@ -8222,16 +8219,16 @@
         <v>1</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="G2" s="19"/>
       <c r="H2" s="18" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="18" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="B3" s="18" t="s">
         <v>228</v>
@@ -8244,16 +8241,16 @@
         <v>2</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="G3" s="19"/>
       <c r="H3" s="18" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="18" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="B4" s="18" t="s">
         <v>228</v>
@@ -8266,11 +8263,11 @@
         <v>3</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="G4" s="19"/>
       <c r="H4" s="18" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -8292,7 +8289,7 @@
       </c>
       <c r="G5" s="19"/>
       <c r="H5" s="18" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -8314,7 +8311,7 @@
       </c>
       <c r="G6" s="19"/>
       <c r="H6" s="18" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -8336,7 +8333,7 @@
       </c>
       <c r="G7" s="19"/>
       <c r="H7" s="18" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -8344,7 +8341,7 @@
         <v>263</v>
       </c>
       <c r="B8" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="C8" t="s">
         <v>86</v>
@@ -8368,7 +8365,7 @@
         <v>263</v>
       </c>
       <c r="B9" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="C9" t="s">
         <v>86</v>
@@ -8392,7 +8389,7 @@
         <v>263</v>
       </c>
       <c r="B10" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="C10" t="s">
         <v>86</v>
@@ -8404,16 +8401,16 @@
         <v>213</v>
       </c>
       <c r="F10" s="21" t="s">
+        <v>467</v>
+      </c>
+      <c r="G10" t="s">
         <v>468</v>
-      </c>
-      <c r="G10" t="s">
-        <v>469</v>
       </c>
       <c r="H10"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="B11" t="s">
         <v>78</v>
@@ -8437,7 +8434,7 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="B12" t="s">
         <v>78</v>
@@ -8461,7 +8458,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="B13" t="s">
         <v>78</v>
@@ -8485,7 +8482,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="B14" t="s">
         <v>78</v>
@@ -8509,7 +8506,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="B15" t="s">
         <v>78</v>
@@ -8524,14 +8521,14 @@
         <v>5</v>
       </c>
       <c r="F15" s="21" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="G15"/>
       <c r="H15"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="B16" t="s">
         <v>208</v>
@@ -8553,7 +8550,7 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="B17" t="s">
         <v>208</v>
@@ -8575,7 +8572,7 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="B18" t="s">
         <v>208</v>
@@ -8597,7 +8594,7 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="B19" t="s">
         <v>208</v>
@@ -8619,7 +8616,7 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="B20" t="s">
         <v>208</v>
@@ -8636,12 +8633,12 @@
       </c>
       <c r="G20"/>
       <c r="H20" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="B21" t="s">
         <v>231</v>
@@ -8654,7 +8651,7 @@
         <v>1</v>
       </c>
       <c r="F21" s="21" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="G21"/>
       <c r="H21"/>
@@ -8663,7 +8660,7 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="B22" t="s">
         <v>231</v>
@@ -8676,7 +8673,7 @@
         <v>2</v>
       </c>
       <c r="F22" s="21" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="G22"/>
       <c r="H22"/>
@@ -8685,7 +8682,7 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="B23" t="s">
         <v>231</v>
@@ -8698,7 +8695,7 @@
         <v>3</v>
       </c>
       <c r="F23" s="21" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="G23"/>
       <c r="H23"/>
@@ -8707,7 +8704,7 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="B24" t="s">
         <v>233</v>
@@ -8724,14 +8721,14 @@
       </c>
       <c r="G24"/>
       <c r="H24" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="I24" s="16"/>
       <c r="J24" s="3"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="B25" t="s">
         <v>233</v>
@@ -8748,14 +8745,14 @@
       </c>
       <c r="G25"/>
       <c r="H25" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="I25" s="15"/>
       <c r="J25" s="4"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="B26" t="s">
         <v>233</v>
@@ -8772,7 +8769,7 @@
       </c>
       <c r="G26"/>
       <c r="H26" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="I26" s="15"/>
       <c r="J26" s="4"/>
@@ -8792,7 +8789,7 @@
         <v>1</v>
       </c>
       <c r="F27" s="21" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="G27"/>
       <c r="H27"/>
@@ -8814,7 +8811,7 @@
         <v>2</v>
       </c>
       <c r="F28" s="21" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="G28"/>
       <c r="H28"/>
@@ -8836,7 +8833,7 @@
         <v>3</v>
       </c>
       <c r="F29" s="21" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="G29"/>
       <c r="H29"/>
@@ -8860,7 +8857,7 @@
       </c>
       <c r="G30"/>
       <c r="H30" s="21" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
@@ -8882,7 +8879,7 @@
       </c>
       <c r="G31"/>
       <c r="H31" s="21" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
@@ -8904,12 +8901,12 @@
       </c>
       <c r="G32"/>
       <c r="H32" s="21" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="B33" t="s">
         <v>77</v>
@@ -8935,7 +8932,7 @@
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="B34" t="s">
         <v>77</v>
@@ -8961,7 +8958,7 @@
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="B35" t="s">
         <v>77</v>
@@ -8987,7 +8984,7 @@
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="B36" t="s">
         <v>77</v>
@@ -9002,13 +8999,13 @@
         <v>214</v>
       </c>
       <c r="F36" s="21" t="s">
+        <v>473</v>
+      </c>
+      <c r="G36" t="s">
         <v>474</v>
       </c>
-      <c r="G36" t="s">
+      <c r="H36" t="s">
         <v>475</v>
-      </c>
-      <c r="H36" t="s">
-        <v>476</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
@@ -9016,7 +9013,7 @@
         <v>265</v>
       </c>
       <c r="B37" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="C37"/>
       <c r="D37" t="s">
@@ -9036,7 +9033,7 @@
         <v>265</v>
       </c>
       <c r="B38" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="C38"/>
       <c r="D38" t="s">
@@ -9056,7 +9053,7 @@
         <v>265</v>
       </c>
       <c r="B39" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="C39"/>
       <c r="D39" t="s">
@@ -9076,17 +9073,17 @@
         <v>265</v>
       </c>
       <c r="B40" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="C40"/>
       <c r="D40" t="s">
         <v>84</v>
       </c>
       <c r="E40" s="21" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="F40" s="21" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="G40"/>
       <c r="H40"/>
@@ -9096,7 +9093,7 @@
         <v>266</v>
       </c>
       <c r="B41" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="C41"/>
       <c r="D41" t="s">
@@ -9118,7 +9115,7 @@
         <v>266</v>
       </c>
       <c r="B42" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="C42"/>
       <c r="D42" t="s">
@@ -9140,14 +9137,14 @@
         <v>266</v>
       </c>
       <c r="B43" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="C43"/>
       <c r="D43" t="s">
         <v>226</v>
       </c>
       <c r="E43" s="21" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="F43" s="21">
         <v>3</v>
@@ -9162,29 +9159,29 @@
         <v>266</v>
       </c>
       <c r="B44" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="C44"/>
       <c r="D44" t="s">
         <v>226</v>
       </c>
       <c r="E44" s="21" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="F44" s="21" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="G44"/>
       <c r="H44" s="21" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
+        <v>478</v>
+      </c>
+      <c r="B45" t="s">
         <v>479</v>
-      </c>
-      <c r="B45" t="s">
-        <v>480</v>
       </c>
       <c r="C45" t="s">
         <v>89</v>
@@ -9207,10 +9204,10 @@
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
+        <v>478</v>
+      </c>
+      <c r="B46" t="s">
         <v>479</v>
-      </c>
-      <c r="B46" t="s">
-        <v>480</v>
       </c>
       <c r="C46" t="s">
         <v>89</v>
@@ -9222,21 +9219,21 @@
         <v>210</v>
       </c>
       <c r="F46" s="21" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="G46" t="s">
+        <v>480</v>
+      </c>
+      <c r="H46" t="s">
         <v>481</v>
-      </c>
-      <c r="H46" t="s">
-        <v>482</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
+        <v>478</v>
+      </c>
+      <c r="B47" t="s">
         <v>479</v>
-      </c>
-      <c r="B47" t="s">
-        <v>480</v>
       </c>
       <c r="C47" t="s">
         <v>89</v>
@@ -9259,10 +9256,10 @@
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
+        <v>478</v>
+      </c>
+      <c r="B48" t="s">
         <v>479</v>
-      </c>
-      <c r="B48" t="s">
-        <v>480</v>
       </c>
       <c r="C48" t="s">
         <v>89</v>
@@ -9288,7 +9285,7 @@
         <v>267</v>
       </c>
       <c r="B49" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="C49" t="s">
         <v>89</v>
@@ -9312,7 +9309,7 @@
         <v>264</v>
       </c>
       <c r="B50" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="C50"/>
       <c r="D50" t="s">
@@ -9336,7 +9333,7 @@
         <v>264</v>
       </c>
       <c r="B51" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="C51"/>
       <c r="D51" t="s">
@@ -9360,7 +9357,7 @@
         <v>103</v>
       </c>
       <c r="B52" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="C52" t="s">
         <v>89</v>
@@ -9385,7 +9382,7 @@
         <v>157</v>
       </c>
       <c r="C53" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="D53" t="s">
         <v>84</v>
@@ -9394,13 +9391,13 @@
         <v>211</v>
       </c>
       <c r="F53" s="21" t="s">
+        <v>434</v>
+      </c>
+      <c r="G53" t="s">
         <v>435</v>
       </c>
-      <c r="G53" t="s">
+      <c r="H53" s="21" t="s">
         <v>436</v>
-      </c>
-      <c r="H53" s="21" t="s">
-        <v>437</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
@@ -9411,7 +9408,7 @@
         <v>157</v>
       </c>
       <c r="C54" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="D54" t="s">
         <v>84</v>
@@ -9420,13 +9417,13 @@
         <v>210</v>
       </c>
       <c r="F54" s="21" t="s">
+        <v>437</v>
+      </c>
+      <c r="G54" t="s">
         <v>438</v>
       </c>
-      <c r="G54" t="s">
+      <c r="H54" s="21" t="s">
         <v>439</v>
-      </c>
-      <c r="H54" s="21" t="s">
-        <v>440</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
@@ -9437,7 +9434,7 @@
         <v>157</v>
       </c>
       <c r="C55" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="D55" t="s">
         <v>84</v>
@@ -9446,13 +9443,13 @@
         <v>213</v>
       </c>
       <c r="F55" s="21" t="s">
+        <v>440</v>
+      </c>
+      <c r="G55" t="s">
         <v>441</v>
       </c>
-      <c r="G55" t="s">
+      <c r="H55" s="21" t="s">
         <v>442</v>
-      </c>
-      <c r="H55" s="21" t="s">
-        <v>443</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
@@ -9463,7 +9460,7 @@
         <v>157</v>
       </c>
       <c r="C56" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="D56" t="s">
         <v>84</v>
@@ -9472,13 +9469,13 @@
         <v>214</v>
       </c>
       <c r="F56" s="21" t="s">
+        <v>443</v>
+      </c>
+      <c r="G56" t="s">
         <v>444</v>
       </c>
-      <c r="G56" t="s">
+      <c r="H56" s="21" t="s">
         <v>445</v>
-      </c>
-      <c r="H56" s="21" t="s">
-        <v>446</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
@@ -9489,7 +9486,7 @@
         <v>157</v>
       </c>
       <c r="C57" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="D57" t="s">
         <v>84</v>
@@ -9498,13 +9495,13 @@
         <v>223</v>
       </c>
       <c r="F57" s="21" t="s">
+        <v>446</v>
+      </c>
+      <c r="G57" t="s">
         <v>447</v>
       </c>
-      <c r="G57" t="s">
+      <c r="H57" s="21" t="s">
         <v>448</v>
-      </c>
-      <c r="H57" s="21" t="s">
-        <v>449</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
@@ -9515,7 +9512,7 @@
         <v>157</v>
       </c>
       <c r="C58" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="D58" t="s">
         <v>84</v>
@@ -9524,13 +9521,13 @@
         <v>222</v>
       </c>
       <c r="F58" s="21" t="s">
+        <v>449</v>
+      </c>
+      <c r="G58" t="s">
         <v>450</v>
       </c>
-      <c r="G58" t="s">
+      <c r="H58" s="21" t="s">
         <v>451</v>
-      </c>
-      <c r="H58" s="21" t="s">
-        <v>452</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
@@ -9541,22 +9538,22 @@
         <v>157</v>
       </c>
       <c r="C59" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="D59" t="s">
         <v>84</v>
       </c>
       <c r="E59" s="21" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="F59" s="21" t="s">
+        <v>452</v>
+      </c>
+      <c r="G59" t="s">
         <v>453</v>
       </c>
-      <c r="G59" t="s">
+      <c r="H59" s="21" t="s">
         <v>454</v>
-      </c>
-      <c r="H59" s="21" t="s">
-        <v>455</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
@@ -9567,7 +9564,7 @@
         <v>157</v>
       </c>
       <c r="C60" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="D60" t="s">
         <v>84</v>
@@ -9576,13 +9573,13 @@
         <v>227</v>
       </c>
       <c r="F60" s="21" t="s">
+        <v>455</v>
+      </c>
+      <c r="G60" t="s">
         <v>456</v>
       </c>
-      <c r="G60" t="s">
+      <c r="H60" s="21" t="s">
         <v>457</v>
-      </c>
-      <c r="H60" s="21" t="s">
-        <v>458</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
@@ -9593,7 +9590,7 @@
         <v>157</v>
       </c>
       <c r="C61" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="D61" t="s">
         <v>84</v>
@@ -9602,13 +9599,13 @@
         <v>212</v>
       </c>
       <c r="F61" s="21" t="s">
+        <v>458</v>
+      </c>
+      <c r="G61" t="s">
         <v>459</v>
       </c>
-      <c r="G61" t="s">
+      <c r="H61" s="21" t="s">
         <v>460</v>
-      </c>
-      <c r="H61" s="21" t="s">
-        <v>461</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
@@ -9619,7 +9616,7 @@
         <v>160</v>
       </c>
       <c r="C62" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="D62" t="s">
         <v>84</v>
@@ -9628,10 +9625,10 @@
         <v>211</v>
       </c>
       <c r="F62" s="21" t="s">
+        <v>434</v>
+      </c>
+      <c r="G62" t="s">
         <v>435</v>
-      </c>
-      <c r="G62" t="s">
-        <v>436</v>
       </c>
       <c r="H62"/>
     </row>
@@ -9643,7 +9640,7 @@
         <v>160</v>
       </c>
       <c r="C63" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="D63" t="s">
         <v>84</v>
@@ -9652,10 +9649,10 @@
         <v>210</v>
       </c>
       <c r="F63" s="21" t="s">
+        <v>437</v>
+      </c>
+      <c r="G63" t="s">
         <v>438</v>
-      </c>
-      <c r="G63" t="s">
-        <v>439</v>
       </c>
       <c r="H63"/>
     </row>
@@ -9667,7 +9664,7 @@
         <v>160</v>
       </c>
       <c r="C64" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="D64" t="s">
         <v>84</v>
@@ -9676,10 +9673,10 @@
         <v>213</v>
       </c>
       <c r="F64" s="21" t="s">
+        <v>440</v>
+      </c>
+      <c r="G64" t="s">
         <v>441</v>
-      </c>
-      <c r="G64" t="s">
-        <v>442</v>
       </c>
       <c r="H64"/>
     </row>
@@ -9691,7 +9688,7 @@
         <v>160</v>
       </c>
       <c r="C65" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="D65" t="s">
         <v>84</v>
@@ -9700,10 +9697,10 @@
         <v>214</v>
       </c>
       <c r="F65" s="21" t="s">
+        <v>443</v>
+      </c>
+      <c r="G65" t="s">
         <v>444</v>
-      </c>
-      <c r="G65" t="s">
-        <v>445</v>
       </c>
       <c r="H65"/>
     </row>
@@ -9715,7 +9712,7 @@
         <v>160</v>
       </c>
       <c r="C66" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="D66" t="s">
         <v>84</v>
@@ -9724,10 +9721,10 @@
         <v>223</v>
       </c>
       <c r="F66" s="21" t="s">
+        <v>446</v>
+      </c>
+      <c r="G66" t="s">
         <v>447</v>
-      </c>
-      <c r="G66" t="s">
-        <v>448</v>
       </c>
       <c r="H66"/>
     </row>
@@ -9739,7 +9736,7 @@
         <v>160</v>
       </c>
       <c r="C67" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="D67" t="s">
         <v>84</v>
@@ -9748,10 +9745,10 @@
         <v>222</v>
       </c>
       <c r="F67" s="21" t="s">
+        <v>449</v>
+      </c>
+      <c r="G67" t="s">
         <v>450</v>
-      </c>
-      <c r="G67" t="s">
-        <v>451</v>
       </c>
       <c r="H67"/>
     </row>
@@ -9763,19 +9760,19 @@
         <v>160</v>
       </c>
       <c r="C68" t="s">
+        <v>461</v>
+      </c>
+      <c r="D68" t="s">
+        <v>84</v>
+      </c>
+      <c r="E68" s="21" t="s">
         <v>462</v>
       </c>
-      <c r="D68" t="s">
-        <v>84</v>
-      </c>
-      <c r="E68" s="21" t="s">
-        <v>463</v>
-      </c>
       <c r="F68" s="21" t="s">
+        <v>452</v>
+      </c>
+      <c r="G68" t="s">
         <v>453</v>
-      </c>
-      <c r="G68" t="s">
-        <v>454</v>
       </c>
       <c r="H68"/>
     </row>
@@ -9787,7 +9784,7 @@
         <v>160</v>
       </c>
       <c r="C69" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="D69" t="s">
         <v>84</v>
@@ -9796,10 +9793,10 @@
         <v>227</v>
       </c>
       <c r="F69" s="21" t="s">
+        <v>455</v>
+      </c>
+      <c r="G69" t="s">
         <v>456</v>
-      </c>
-      <c r="G69" t="s">
-        <v>457</v>
       </c>
       <c r="H69"/>
     </row>
@@ -9811,7 +9808,7 @@
         <v>160</v>
       </c>
       <c r="C70" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="D70" t="s">
         <v>84</v>
@@ -9820,10 +9817,10 @@
         <v>212</v>
       </c>
       <c r="F70" s="21" t="s">
+        <v>458</v>
+      </c>
+      <c r="G70" t="s">
         <v>459</v>
-      </c>
-      <c r="G70" t="s">
-        <v>460</v>
       </c>
       <c r="H70"/>
     </row>
@@ -9846,7 +9843,7 @@
       </c>
       <c r="G71"/>
       <c r="H71" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.25">
@@ -9868,7 +9865,7 @@
       </c>
       <c r="G72"/>
       <c r="H72" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.25">
@@ -9890,7 +9887,7 @@
       </c>
       <c r="G73"/>
       <c r="H73" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.25">
@@ -9912,7 +9909,7 @@
       </c>
       <c r="G74"/>
       <c r="H74" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.25">
@@ -9934,7 +9931,7 @@
       </c>
       <c r="G75"/>
       <c r="H75" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.25">
@@ -9956,7 +9953,7 @@
       </c>
       <c r="G76"/>
       <c r="H76" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.25">
@@ -9971,14 +9968,14 @@
         <v>226</v>
       </c>
       <c r="E77" s="21" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="F77" s="21" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="G77"/>
       <c r="H77" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.25">
@@ -10000,7 +9997,7 @@
       </c>
       <c r="G78"/>
       <c r="H78" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.25">
@@ -10022,7 +10019,7 @@
       </c>
       <c r="G79"/>
       <c r="H79" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.25">
@@ -10392,492 +10389,492 @@
     </row>
     <row r="2" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
+        <v>485</v>
+      </c>
+      <c r="B2" s="12" t="s">
         <v>486</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="C2" s="12" t="s">
         <v>487</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="D2" s="12" t="s">
         <v>488</v>
-      </c>
-      <c r="D2" s="12" t="s">
-        <v>489</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
+        <v>489</v>
+      </c>
+      <c r="B3" s="12" t="s">
         <v>490</v>
       </c>
-      <c r="B3" s="12" t="s">
-        <v>491</v>
-      </c>
       <c r="C3" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B4" s="12" t="s">
+        <v>491</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>487</v>
+      </c>
+      <c r="D4" s="12" t="s">
         <v>492</v>
-      </c>
-      <c r="C4" s="12" t="s">
-        <v>488</v>
-      </c>
-      <c r="D4" s="12" t="s">
-        <v>493</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B13" s="12" t="s">
+        <v>500</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>487</v>
+      </c>
+      <c r="D13" s="12" t="s">
         <v>501</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>488</v>
-      </c>
-      <c r="D13" s="12" t="s">
-        <v>502</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="B14" s="12" t="s">
+        <v>502</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>487</v>
+      </c>
+      <c r="D14" s="12" t="s">
         <v>503</v>
-      </c>
-      <c r="C14" s="12" t="s">
-        <v>488</v>
-      </c>
-      <c r="D14" s="12" t="s">
-        <v>504</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B15" s="12" t="s">
+        <v>504</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>487</v>
+      </c>
+      <c r="D15" s="12" t="s">
         <v>505</v>
-      </c>
-      <c r="C15" s="12" t="s">
-        <v>488</v>
-      </c>
-      <c r="D15" s="12" t="s">
-        <v>506</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="135" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B16" s="12" t="s">
+        <v>506</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>487</v>
+      </c>
+      <c r="D16" s="12" t="s">
         <v>507</v>
-      </c>
-      <c r="C16" s="12" t="s">
-        <v>488</v>
-      </c>
-      <c r="D16" s="12" t="s">
-        <v>508</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="120" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="B17" s="12" t="s">
+        <v>508</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>487</v>
+      </c>
+      <c r="D17" s="12" t="s">
         <v>509</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>488</v>
-      </c>
-      <c r="D17" s="12" t="s">
-        <v>510</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="90" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="195" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="B20" s="12" t="s">
+        <v>512</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>487</v>
+      </c>
+      <c r="D20" s="12" t="s">
         <v>513</v>
-      </c>
-      <c r="C20" s="12" t="s">
-        <v>488</v>
-      </c>
-      <c r="D20" s="12" t="s">
-        <v>514</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="270" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D23" s="12" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="90" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="B24" s="12" t="s">
+        <v>517</v>
+      </c>
+      <c r="C24" s="12" t="s">
+        <v>487</v>
+      </c>
+      <c r="D24" s="12" t="s">
         <v>518</v>
-      </c>
-      <c r="C24" s="12" t="s">
-        <v>488</v>
-      </c>
-      <c r="D24" s="12" t="s">
-        <v>519</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A26" s="12" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="12" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B27" s="12" t="s">
+        <v>521</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>487</v>
+      </c>
+      <c r="D27" s="12" t="s">
         <v>522</v>
-      </c>
-      <c r="C27" s="12" t="s">
-        <v>488</v>
-      </c>
-      <c r="D27" s="12" t="s">
-        <v>523</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="135" x14ac:dyDescent="0.25">
       <c r="A28" s="12" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="B28" s="12" t="s">
+        <v>523</v>
+      </c>
+      <c r="C28" s="12" t="s">
+        <v>487</v>
+      </c>
+      <c r="D28" s="12" t="s">
         <v>524</v>
-      </c>
-      <c r="C28" s="12" t="s">
-        <v>488</v>
-      </c>
-      <c r="D28" s="12" t="s">
-        <v>525</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="12" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="B29" s="12" t="s">
+        <v>525</v>
+      </c>
+      <c r="C29" s="12" t="s">
+        <v>487</v>
+      </c>
+      <c r="D29" s="12" t="s">
         <v>526</v>
-      </c>
-      <c r="C29" s="12" t="s">
-        <v>488</v>
-      </c>
-      <c r="D29" s="12" t="s">
-        <v>527</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A30" s="12" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="B30" s="12" t="s">
+        <v>527</v>
+      </c>
+      <c r="C30" s="12" t="s">
+        <v>487</v>
+      </c>
+      <c r="D30" s="12" t="s">
         <v>528</v>
-      </c>
-      <c r="C30" s="12" t="s">
-        <v>488</v>
-      </c>
-      <c r="D30" s="12" t="s">
-        <v>529</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="B31" s="12" t="s">
+        <v>529</v>
+      </c>
+      <c r="C31" s="12" t="s">
+        <v>487</v>
+      </c>
+      <c r="D31" s="12" t="s">
         <v>530</v>
-      </c>
-      <c r="C31" s="12" t="s">
-        <v>488</v>
-      </c>
-      <c r="D31" s="12" t="s">
-        <v>531</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="B32" s="12" t="s">
+        <v>531</v>
+      </c>
+      <c r="C32" s="12" t="s">
+        <v>487</v>
+      </c>
+      <c r="D32" s="12" t="s">
         <v>532</v>
-      </c>
-      <c r="C32" s="12" t="s">
-        <v>488</v>
-      </c>
-      <c r="D32" s="12" t="s">
-        <v>533</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" s="12" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="B33" s="12" t="s">
+        <v>533</v>
+      </c>
+      <c r="C33" s="12" t="s">
+        <v>487</v>
+      </c>
+      <c r="D33" s="12" t="s">
         <v>534</v>
-      </c>
-      <c r="C33" s="12" t="s">
-        <v>488</v>
-      </c>
-      <c r="D33" s="12" t="s">
-        <v>535</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="12" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="B34" s="12" t="s">
+        <v>535</v>
+      </c>
+      <c r="C34" s="12" t="s">
+        <v>487</v>
+      </c>
+      <c r="D34" s="12" t="s">
         <v>536</v>
-      </c>
-      <c r="C34" s="12" t="s">
-        <v>488</v>
-      </c>
-      <c r="D34" s="12" t="s">
-        <v>537</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="195" x14ac:dyDescent="0.25">
       <c r="A35" s="12" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="C35" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="105" x14ac:dyDescent="0.25">
       <c r="A36" s="12" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D36" s="12" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="45" x14ac:dyDescent="0.25">
@@ -10885,13 +10882,13 @@
         <v>378</v>
       </c>
       <c r="B37" s="12" t="s">
+        <v>539</v>
+      </c>
+      <c r="C37" s="12" t="s">
+        <v>487</v>
+      </c>
+      <c r="D37" s="12" t="s">
         <v>540</v>
-      </c>
-      <c r="C37" s="12" t="s">
-        <v>488</v>
-      </c>
-      <c r="D37" s="12" t="s">
-        <v>541</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="90" x14ac:dyDescent="0.25">
@@ -10899,13 +10896,13 @@
         <v>300</v>
       </c>
       <c r="B38" s="12" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D38" s="12" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="90" x14ac:dyDescent="0.25">
@@ -10916,10 +10913,10 @@
         <v>292</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="105" x14ac:dyDescent="0.25">
@@ -10930,10 +10927,10 @@
         <v>291</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D40" s="12" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="45" x14ac:dyDescent="0.25">
@@ -10944,10 +10941,10 @@
         <v>297</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="45" x14ac:dyDescent="0.25">
@@ -10958,10 +10955,10 @@
         <v>298</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D42" s="12" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="45" x14ac:dyDescent="0.25">
@@ -10972,10 +10969,10 @@
         <v>293</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="45" x14ac:dyDescent="0.25">
@@ -10986,10 +10983,10 @@
         <v>295</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D44" s="12" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="45" x14ac:dyDescent="0.25">
@@ -11000,10 +10997,10 @@
         <v>294</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D45" s="12" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="60" x14ac:dyDescent="0.25">
@@ -11014,10 +11011,10 @@
         <v>285</v>
       </c>
       <c r="C46" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D46" s="12" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="120" x14ac:dyDescent="0.25">
@@ -11028,10 +11025,10 @@
         <v>136</v>
       </c>
       <c r="C47" s="12" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="D47" s="12" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="135" x14ac:dyDescent="0.25">
@@ -11042,10 +11039,10 @@
         <v>137</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="D48" s="12" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
     </row>
     <row r="49" spans="1:9" ht="75" x14ac:dyDescent="0.25">
@@ -11056,10 +11053,10 @@
         <v>277</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D49" s="12" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="50" spans="1:9" ht="60" x14ac:dyDescent="0.25">
@@ -11070,10 +11067,10 @@
         <v>281</v>
       </c>
       <c r="C50" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D50" s="12" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
     </row>
     <row r="51" spans="1:9" ht="45" x14ac:dyDescent="0.25">
@@ -11084,24 +11081,24 @@
         <v>301</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D51" s="12" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
     </row>
     <row r="52" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A52" s="12" t="s">
+        <v>596</v>
+      </c>
+      <c r="B52" s="12" t="s">
+        <v>596</v>
+      </c>
+      <c r="C52" s="12" t="s">
+        <v>487</v>
+      </c>
+      <c r="D52" s="12" t="s">
         <v>597</v>
-      </c>
-      <c r="B52" s="12" t="s">
-        <v>597</v>
-      </c>
-      <c r="C52" s="12" t="s">
-        <v>488</v>
-      </c>
-      <c r="D52" s="12" t="s">
-        <v>598</v>
       </c>
     </row>
     <row r="53" spans="1:9" ht="45" x14ac:dyDescent="0.25">
@@ -11112,10 +11109,10 @@
         <v>303</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D53" s="12" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
     </row>
     <row r="54" spans="1:9" ht="45" x14ac:dyDescent="0.25">
@@ -11126,10 +11123,10 @@
         <v>304</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D54" s="12" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
     </row>
     <row r="55" spans="1:9" ht="90" x14ac:dyDescent="0.25">
@@ -11140,10 +11137,10 @@
         <v>305</v>
       </c>
       <c r="C55" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D55" s="12" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -11154,10 +11151,10 @@
         <v>306</v>
       </c>
       <c r="C56" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D56" s="12" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
     <row r="57" spans="1:9" ht="135" x14ac:dyDescent="0.25">
@@ -11168,10 +11165,10 @@
         <v>307</v>
       </c>
       <c r="C57" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D57" s="12" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="58" spans="1:9" ht="75" x14ac:dyDescent="0.25">
@@ -11182,10 +11179,10 @@
         <v>308</v>
       </c>
       <c r="C58" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D58" s="12" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="59" spans="1:9" ht="75" x14ac:dyDescent="0.25">
@@ -11196,10 +11193,10 @@
         <v>309</v>
       </c>
       <c r="C59" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D59" s="12" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="60" spans="1:9" ht="120" x14ac:dyDescent="0.25">
@@ -11210,10 +11207,10 @@
         <v>310</v>
       </c>
       <c r="C60" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D60" s="12" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="61" spans="1:9" ht="75" x14ac:dyDescent="0.25">
@@ -11224,10 +11221,10 @@
         <v>311</v>
       </c>
       <c r="C61" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D61" s="12" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="62" spans="1:9" ht="75" x14ac:dyDescent="0.25">
@@ -11238,24 +11235,24 @@
         <v>379</v>
       </c>
       <c r="C62" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D62" s="12" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="63" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A63" s="12" t="s">
+        <v>588</v>
+      </c>
+      <c r="B63" s="12" t="s">
+        <v>588</v>
+      </c>
+      <c r="C63" s="12" t="s">
+        <v>487</v>
+      </c>
+      <c r="D63" s="12" t="s">
         <v>589</v>
-      </c>
-      <c r="B63" s="12" t="s">
-        <v>589</v>
-      </c>
-      <c r="C63" s="12" t="s">
-        <v>488</v>
-      </c>
-      <c r="D63" s="12" t="s">
-        <v>590</v>
       </c>
       <c r="I63"/>
     </row>
@@ -11267,210 +11264,210 @@
         <v>284</v>
       </c>
       <c r="C64" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D64" s="12" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="I64"/>
     </row>
     <row r="65" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A65" s="12" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="B65" s="12" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="C65" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D65" s="12" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="I65"/>
     </row>
     <row r="66" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A66" s="12" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="B66" s="12" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="C66" s="12" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="D66" s="12" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="I66"/>
     </row>
     <row r="67" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A67" s="12" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="B67" s="12" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="C67" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D67" s="12" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="I67"/>
     </row>
     <row r="68" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A68" s="12" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B68" s="12" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="C68" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D68" s="12" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
     </row>
     <row r="69" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A69" s="12" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B69" s="12" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="C69" s="12" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="D69" s="12" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
     </row>
     <row r="70" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A70" s="12" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="B70" s="12" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="C70" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D70" s="12" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="71" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A71" s="12" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="B71" s="12" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="C71" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D71" s="12" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" s="12" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B72" s="12" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="C72" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D72" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
     </row>
     <row r="73" spans="1:9" ht="120" x14ac:dyDescent="0.25">
       <c r="A73" s="12" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="B73" s="12" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="C73" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D73" s="12" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
     </row>
     <row r="74" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A74" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="B74" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="C74" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D74" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
     </row>
     <row r="75" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A75" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="B75" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="C75" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D75" s="12" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
     </row>
     <row r="76" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A76" s="12" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="B76" s="12" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="C76" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D76" s="12" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
     </row>
     <row r="77" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A77" s="12" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B77" s="12" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="C77" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D77" s="12" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
     </row>
     <row r="78" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A78" s="12" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="B78" s="12" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="C78" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D78" s="12" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
     </row>
   </sheetData>

</xml_diff>